<commit_message>
docs(entrega): textos analiticos finais 3.1/3.2/3.3 + checklist final (Fase 8)
- output/textos_analiticos.md: redacao final respondendo 3.1.a/b, 3.2.a/b/c, 3.3.a/b/c
- Checklist final do docs/03 marcado (9/9): dados TCE-RS, auditoria, notebooks
  rodando, tabelas/graficos exportados com fonte, nominal/real, deflator, perguntas
- 4 notebooks (00/31/32/33) reexecutados de ponta a ponta com nbconvert (0 erros);
  planilhas regeradas (timestamp da aba Metadados)
- TAREFAS.md: Fase 8 concluida (projeto - parte do Vitor - encerrado)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/tabelas/3_3_maiores_credores_2024.xlsx
+++ b/output/tabelas/3_3_maiores_credores_2024.xlsx
@@ -1730,127 +1730,127 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>306</t>
+          <t>10699</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>INSTITUTO DE PREVIDENCIA DO ESTADO DO RS</t>
+          <t>EPTV - EMPRESA PUBLICA DE TRANSITO DE VIAMAO S/A</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Previdencia estadual (IPE-RS)</t>
+          <t>Empresa publica propria (EPTV)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Regime proprio estadual - encargo</t>
+          <t>Empresa publica municipal de transito - repasse interno</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>11310</t>
+          <t>814</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>IPREV - INST DE PREVIDENCIA DOS SERV. DE VIAMAO</t>
+          <t>FOLHA DE PAGAMENTO</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Previdencia propria (IPREV)</t>
+          <t>Folha de pagamento</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Autarquia previdenciaria do proprio municipio (RPPS)</t>
+          <t>Pessoal/servidores - nao e contratacao de fornecedor</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>13285</t>
+          <t>511</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SECRETARIA DA RECEITA FEDERAL</t>
+          <t>TRIBUNAL REGIONAL DO TRABALHO 4A REGIAO</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Tributo federal (Receita Federal)</t>
+          <t>Deposito judicial (TRT-4)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Recolhimento de tributos/retencoes</t>
+          <t>Consignacoes/depositos judiciais</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>7243</t>
+          <t>304</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>3A VARA CIVEL DA COMARCA DE VIAMAO</t>
+          <t>SEFAZ/RS</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Deposito judicial (Vara Civel Viamao)</t>
+          <t>Tributo estadual (SEFAZ/RS)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Consignacoes/depositos judiciais</t>
+          <t>Recolhimento de tributos estaduais</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>6400</t>
+          <t>13755</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>TRIBUNAL DE JUSTICA DO ESTADO DO RGS</t>
+          <t>BRDE - BANCO REGIONAL DE DESENV DO EXTREMO SUL</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Deposito judicial (TJ-RS)</t>
+          <t>Servico da divida (BRDE)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Consignacoes/depositos judiciais</t>
+          <t>Amortizacao/juros de emprestimo - nao e fornecedor</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>252</t>
+          <t>6400</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>PODER JUDICIARIO</t>
+          <t>TRIBUNAL DE JUSTICA DO ESTADO DO RGS</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Deposito judicial (Poder Judiciario)</t>
+          <t>Deposito judicial (TJ-RS)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1862,132 +1862,132 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>13755</t>
+          <t>7243</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>BRDE - BANCO REGIONAL DE DESENV DO EXTREMO SUL</t>
+          <t>3A VARA CIVEL DA COMARCA DE VIAMAO</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Servico da divida (BRDE)</t>
+          <t>Deposito judicial (Vara Civel Viamao)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Amortizacao/juros de emprestimo - nao e fornecedor</t>
+          <t>Consignacoes/depositos judiciais</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>511</t>
+          <t>11310</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>TRIBUNAL REGIONAL DO TRABALHO 4A REGIAO</t>
+          <t>IPREV - INST DE PREVIDENCIA DOS SERV. DE VIAMAO</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Deposito judicial (TRT-4)</t>
+          <t>Previdencia propria (IPREV)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Consignacoes/depositos judiciais</t>
+          <t>Autarquia previdenciaria do proprio municipio (RPPS)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>304</t>
+          <t>122</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>SEFAZ/RS</t>
+          <t>INSS INSTNACSEGDE SOCIAL</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Tributo estadual (SEFAZ/RS)</t>
+          <t>Previdencia federal (INSS)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Recolhimento de tributos estaduais</t>
+          <t>Contribuicao previdenciaria/encargo federal</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>10699</t>
+          <t>252</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>EPTV - EMPRESA PUBLICA DE TRANSITO DE VIAMAO S/A</t>
+          <t>PODER JUDICIARIO</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Empresa publica propria (EPTV)</t>
+          <t>Deposito judicial (Poder Judiciario)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Empresa publica municipal de transito - repasse interno</t>
+          <t>Consignacoes/depositos judiciais</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>814</t>
+          <t>306</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>FOLHA DE PAGAMENTO</t>
+          <t>INSTITUTO DE PREVIDENCIA DO ESTADO DO RS</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Folha de pagamento</t>
+          <t>Previdencia estadual (IPE-RS)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Pessoal/servidores - nao e contratacao de fornecedor</t>
+          <t>Regime proprio estadual - encargo</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>122</t>
+          <t>13285</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>INSS INSTNACSEGDE SOCIAL</t>
+          <t>SECRETARIA DA RECEITA FEDERAL</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Previdencia federal (INSS)</t>
+          <t>Tributo federal (Receita Federal)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Contribuicao previdenciaria/encargo federal</t>
+          <t>Recolhimento de tributos/retencoes</t>
         </is>
       </c>
     </row>
@@ -2175,7 +2175,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-02T22:00:09</t>
+          <t>2026-07-02T22:05:55</t>
         </is>
       </c>
     </row>

</xml_diff>